<commit_message>
Week2: era analysis, CAGR, anomalies - COVID hit growth not margin
</commit_message>
<xml_diff>
--- a/data/TITAN PROJECT.xlsx
+++ b/data/TITAN PROJECT.xlsx
@@ -17,6 +17,8 @@
     <sheet name="Python Output" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Python Summary" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Sheet1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Week2 Pipeline" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Week2 Era Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="IQ_CH">110000</definedName>
@@ -926,6 +928,2208 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:BF11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>raw_material_cost</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>change_in_inventory</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>power_fuel</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>other_mfr_exp</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>employee_cost</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>selling_admin</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>other_expenses</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>other_income</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>depreciation</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ebt</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>net_profit</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>dividend_amount</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>equity_share_cap</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>total_debt</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>total_assets</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>equity_shares</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>reserves</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>debt</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>fixed_assets</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>debtors</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>cash_operating</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>payables</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>cogs</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ebit</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>sales_growth</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>ebitda_growth</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>ebit_growth</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>net_profit_growth</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>gross_profit</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>gross_margin</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>ebitda_margin</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>ebit_margin</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>ebt_margin</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>net_margin</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>avg_debtors</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>debtor_turnover</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>inventory_turnover</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>creditor_turnover</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>fixed_asset_turnover</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>capital_employed</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>capital_turnover</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>debtor_days</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>payables_days</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>inventory_days</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>cash_conversion_cycle</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>roce</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>interest_coverage</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>debt_to_ebitda</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>credit</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>era</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>roce_flag</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>cash_conversion_cycle_flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B2" t="n">
+        <v>13260.83</v>
+      </c>
+      <c r="C2" t="n">
+        <v>9821.139999999999</v>
+      </c>
+      <c r="D2" t="n">
+        <v>313.71</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.84</v>
+      </c>
+      <c r="F2" t="n">
+        <v>160.42</v>
+      </c>
+      <c r="G2" t="n">
+        <v>894.3200000000001</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1211.16</v>
+      </c>
+      <c r="I2" t="n">
+        <v>279.76</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-42.38</v>
+      </c>
+      <c r="K2" t="n">
+        <v>110.53</v>
+      </c>
+      <c r="L2" t="n">
+        <v>37.74</v>
+      </c>
+      <c r="M2" t="n">
+        <v>973.25</v>
+      </c>
+      <c r="N2" t="n">
+        <v>275.97</v>
+      </c>
+      <c r="O2" t="n">
+        <v>711.47</v>
+      </c>
+      <c r="P2" t="n">
+        <v>230.83</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="R2" t="n">
+        <v>8407.57</v>
+      </c>
+      <c r="S2" t="n">
+        <v>8407.57</v>
+      </c>
+      <c r="T2" t="n">
+        <v>887786160</v>
+      </c>
+      <c r="U2" t="n">
+        <v>4143.6</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1882.43</v>
+      </c>
+      <c r="W2" t="n">
+        <v>1188.72</v>
+      </c>
+      <c r="X2" t="n">
+        <v>207.6</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>4925.74</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1712.3</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2292.76</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>10606.01</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>1163.9</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>1053.37</v>
+      </c>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="n">
+        <v>2654.82</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0.2002</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0.0878</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0.0794</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0.07340000000000001</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0.0537</v>
+      </c>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>6114.81</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="n">
+        <v>63</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>136</v>
+      </c>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="n">
+        <v>0.1723</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>27.91</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>Pre-COVID</t>
+        </is>
+      </c>
+      <c r="BE2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B3" t="n">
+        <v>16119.77</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12664.83</v>
+      </c>
+      <c r="D3" t="n">
+        <v>978.61</v>
+      </c>
+      <c r="E3" t="n">
+        <v>45.32</v>
+      </c>
+      <c r="F3" t="n">
+        <v>124.83</v>
+      </c>
+      <c r="G3" t="n">
+        <v>906.26</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1277.81</v>
+      </c>
+      <c r="I3" t="n">
+        <v>435.13</v>
+      </c>
+      <c r="J3" t="n">
+        <v>69.93000000000001</v>
+      </c>
+      <c r="K3" t="n">
+        <v>131.43</v>
+      </c>
+      <c r="L3" t="n">
+        <v>52.92</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1529.78</v>
+      </c>
+      <c r="N3" t="n">
+        <v>427.87</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1130.09</v>
+      </c>
+      <c r="P3" t="n">
+        <v>332.92</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="R3" t="n">
+        <v>9521.040000000001</v>
+      </c>
+      <c r="S3" t="n">
+        <v>9521.040000000001</v>
+      </c>
+      <c r="T3" t="n">
+        <v>887786160</v>
+      </c>
+      <c r="U3" t="n">
+        <v>5001.1</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1691.01</v>
+      </c>
+      <c r="W3" t="n">
+        <v>1473.81</v>
+      </c>
+      <c r="X3" t="n">
+        <v>295.69</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>5924.84</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>-51.12</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>2740.15</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>12762.63</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>1644.200000000001</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>1512.770000000001</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0.2156</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0.4127</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0.4361</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>0.5884</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>3357.140000000001</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>0.2083</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0.09379999999999999</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>0.0949</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>0.0701</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>251.645</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>64.06</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>6780.89</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>62</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>134</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>78</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>0.2231</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>28.59</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>Healthy</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>Pre-COVID</t>
+        </is>
+      </c>
+      <c r="BE3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B4" t="n">
+        <v>19778.52</v>
+      </c>
+      <c r="C4" t="n">
+        <v>15170.66</v>
+      </c>
+      <c r="D4" t="n">
+        <v>776.41</v>
+      </c>
+      <c r="E4" t="n">
+        <v>48.51</v>
+      </c>
+      <c r="F4" t="n">
+        <v>193.28</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1024.44</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1454.32</v>
+      </c>
+      <c r="I4" t="n">
+        <v>669.9299999999999</v>
+      </c>
+      <c r="J4" t="n">
+        <v>178.48</v>
+      </c>
+      <c r="K4" t="n">
+        <v>162.84</v>
+      </c>
+      <c r="L4" t="n">
+        <v>52.54</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1956.89</v>
+      </c>
+      <c r="N4" t="n">
+        <v>568.24</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1404.15</v>
+      </c>
+      <c r="P4" t="n">
+        <v>443.9</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>88.78</v>
+      </c>
+      <c r="R4" t="n">
+        <v>11709.84</v>
+      </c>
+      <c r="S4" t="n">
+        <v>11709.84</v>
+      </c>
+      <c r="T4" t="n">
+        <v>887786160</v>
+      </c>
+      <c r="U4" t="n">
+        <v>5981.37</v>
+      </c>
+      <c r="V4" t="n">
+        <v>2392.98</v>
+      </c>
+      <c r="W4" t="n">
+        <v>1566.63</v>
+      </c>
+      <c r="X4" t="n">
+        <v>420.45</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>7038.82</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>1242.92</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>3246.71</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>15660.48</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>1993.790000000001</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>1830.950000000001</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.2126</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.2103</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0.2425</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>4118.040000000001</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0.2082</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0.1008</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0.0926</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>0.0989</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>358.07</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>55.24</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>12.62</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>8463.129999999999</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>7</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>60</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>130</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>77</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>0.2163</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>34.85</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>Healthy</t>
+        </is>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>Pre-COVID</t>
+        </is>
+      </c>
+      <c r="BE4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B5" t="n">
+        <v>21052</v>
+      </c>
+      <c r="C5" t="n">
+        <v>16033</v>
+      </c>
+      <c r="D5" t="n">
+        <v>878</v>
+      </c>
+      <c r="E5" t="n">
+        <v>52</v>
+      </c>
+      <c r="F5" t="n">
+        <v>215</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1204</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1470</v>
+      </c>
+      <c r="I5" t="n">
+        <v>493</v>
+      </c>
+      <c r="J5" t="n">
+        <v>153</v>
+      </c>
+      <c r="K5" t="n">
+        <v>348</v>
+      </c>
+      <c r="L5" t="n">
+        <v>166</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2102</v>
+      </c>
+      <c r="N5" t="n">
+        <v>609</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1501</v>
+      </c>
+      <c r="P5" t="n">
+        <v>356</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>89</v>
+      </c>
+      <c r="R5" t="n">
+        <v>13544</v>
+      </c>
+      <c r="S5" t="n">
+        <v>13544</v>
+      </c>
+      <c r="T5" t="n">
+        <v>887786160</v>
+      </c>
+      <c r="U5" t="n">
+        <v>6580</v>
+      </c>
+      <c r="V5" t="n">
+        <v>3562</v>
+      </c>
+      <c r="W5" t="n">
+        <v>2633</v>
+      </c>
+      <c r="X5" t="n">
+        <v>312</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>8103</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>-348</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>3313</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>16626</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>2463</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>2115</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0.0644</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0.2353</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0.1551</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>4426</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>0.2102</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>0.1005</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>0.0998</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>0.0713</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>366.225</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>57.48</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>8</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>10231</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>57</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>140</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>89</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>0.2067</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>12.74</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>Healthy</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>COVID</t>
+        </is>
+      </c>
+      <c r="BE5" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B6" t="n">
+        <v>21644</v>
+      </c>
+      <c r="C6" t="n">
+        <v>16292</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-122</v>
+      </c>
+      <c r="E6" t="n">
+        <v>37</v>
+      </c>
+      <c r="F6" t="n">
+        <v>141</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1069</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1029</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1229</v>
+      </c>
+      <c r="J6" t="n">
+        <v>180</v>
+      </c>
+      <c r="K6" t="n">
+        <v>375</v>
+      </c>
+      <c r="L6" t="n">
+        <v>203</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1327</v>
+      </c>
+      <c r="N6" t="n">
+        <v>353</v>
+      </c>
+      <c r="O6" t="n">
+        <v>973</v>
+      </c>
+      <c r="P6" t="n">
+        <v>356</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>89</v>
+      </c>
+      <c r="R6" t="n">
+        <v>16444</v>
+      </c>
+      <c r="S6" t="n">
+        <v>16444</v>
+      </c>
+      <c r="T6" t="n">
+        <v>887786160</v>
+      </c>
+      <c r="U6" t="n">
+        <v>7408</v>
+      </c>
+      <c r="V6" t="n">
+        <v>5638</v>
+      </c>
+      <c r="W6" t="n">
+        <v>2523</v>
+      </c>
+      <c r="X6" t="n">
+        <v>366</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>8408</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>4139</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>3309</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>17661</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>1725</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0.0281</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>-0.2996</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>-0.3617</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>-0.3518</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>3983</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.07969999999999999</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0.0624</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>0.0613</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>339</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>63.85</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>13135</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>56</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>142</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>92</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>0.1028</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>COVID</t>
+        </is>
+      </c>
+      <c r="BE6" t="b">
+        <v>1</v>
+      </c>
+      <c r="BF6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B7" t="n">
+        <v>28799</v>
+      </c>
+      <c r="C7" t="n">
+        <v>26436</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4795</v>
+      </c>
+      <c r="E7" t="n">
+        <v>45</v>
+      </c>
+      <c r="F7" t="n">
+        <v>183</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1356</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1697</v>
+      </c>
+      <c r="I7" t="n">
+        <v>533</v>
+      </c>
+      <c r="J7" t="n">
+        <v>177</v>
+      </c>
+      <c r="K7" t="n">
+        <v>399</v>
+      </c>
+      <c r="L7" t="n">
+        <v>218</v>
+      </c>
+      <c r="M7" t="n">
+        <v>2904</v>
+      </c>
+      <c r="N7" t="n">
+        <v>706</v>
+      </c>
+      <c r="O7" t="n">
+        <v>2173</v>
+      </c>
+      <c r="P7" t="n">
+        <v>667.5</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>89</v>
+      </c>
+      <c r="R7" t="n">
+        <v>21188</v>
+      </c>
+      <c r="S7" t="n">
+        <v>21188</v>
+      </c>
+      <c r="T7" t="n">
+        <v>887786160</v>
+      </c>
+      <c r="U7" t="n">
+        <v>9214</v>
+      </c>
+      <c r="V7" t="n">
+        <v>7275</v>
+      </c>
+      <c r="W7" t="n">
+        <v>2544</v>
+      </c>
+      <c r="X7" t="n">
+        <v>565</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>13609</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>-724</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>4610</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>23225</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>3344</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>2945</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0.3306</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0.9386</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>1.1815</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>1.2333</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>5574</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0.1935</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.1161</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0.1023</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0.1008</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0.0755</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>465.5</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>61.87</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>16578</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>58</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>172</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>120</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>13.51</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="BE7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B8" t="n">
+        <v>40575</v>
+      </c>
+      <c r="C8" t="n">
+        <v>32589</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2234</v>
+      </c>
+      <c r="E8" t="n">
+        <v>59</v>
+      </c>
+      <c r="F8" t="n">
+        <v>225</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1656</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2715</v>
+      </c>
+      <c r="I8" t="n">
+        <v>683</v>
+      </c>
+      <c r="J8" t="n">
+        <v>306</v>
+      </c>
+      <c r="K8" t="n">
+        <v>441</v>
+      </c>
+      <c r="L8" t="n">
+        <v>300</v>
+      </c>
+      <c r="M8" t="n">
+        <v>4447</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1173</v>
+      </c>
+      <c r="O8" t="n">
+        <v>3250</v>
+      </c>
+      <c r="P8" t="n">
+        <v>890</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>89</v>
+      </c>
+      <c r="R8" t="n">
+        <v>27020</v>
+      </c>
+      <c r="S8" t="n">
+        <v>27020</v>
+      </c>
+      <c r="T8" t="n">
+        <v>890000000</v>
+      </c>
+      <c r="U8" t="n">
+        <v>11762</v>
+      </c>
+      <c r="V8" t="n">
+        <v>9367</v>
+      </c>
+      <c r="W8" t="n">
+        <v>2998</v>
+      </c>
+      <c r="X8" t="n">
+        <v>674</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>16584</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>1370</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>5802</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>32295</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>4882</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>4441</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0.4089</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0.4599</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0.508</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0.4956</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>8280</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0.2041</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.1203</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0.1095</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0.1096</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>0.0801</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>619.5</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>21218</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>52</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>149</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>103</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>0.2093</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="BE8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B9" t="n">
+        <v>51084</v>
+      </c>
+      <c r="C9" t="n">
+        <v>42103</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2671</v>
+      </c>
+      <c r="E9" t="n">
+        <v>71</v>
+      </c>
+      <c r="F9" t="n">
+        <v>286</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1875</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3249</v>
+      </c>
+      <c r="I9" t="n">
+        <v>879</v>
+      </c>
+      <c r="J9" t="n">
+        <v>534</v>
+      </c>
+      <c r="K9" t="n">
+        <v>584</v>
+      </c>
+      <c r="L9" t="n">
+        <v>619</v>
+      </c>
+      <c r="M9" t="n">
+        <v>4623</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1127</v>
+      </c>
+      <c r="O9" t="n">
+        <v>3496</v>
+      </c>
+      <c r="P9" t="n">
+        <v>979</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>89</v>
+      </c>
+      <c r="R9" t="n">
+        <v>31547</v>
+      </c>
+      <c r="S9" t="n">
+        <v>31547</v>
+      </c>
+      <c r="T9" t="n">
+        <v>890000000</v>
+      </c>
+      <c r="U9" t="n">
+        <v>9304</v>
+      </c>
+      <c r="V9" t="n">
+        <v>15528</v>
+      </c>
+      <c r="W9" t="n">
+        <v>3709</v>
+      </c>
+      <c r="X9" t="n">
+        <v>1018</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>19051</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>1695</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>6626</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>41664</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>5292</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>4708</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0.0601</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0.0757</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>9420</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0.1844</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.1036</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.0922</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0.0905</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>0.0684</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>846</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>60.38</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>7.71</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>13.77</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>24921</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>47</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>136</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>95</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>0.1889</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="BE9" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B10" t="n">
+        <v>60456</v>
+      </c>
+      <c r="C10" t="n">
+        <v>55271</v>
+      </c>
+      <c r="D10" t="n">
+        <v>7815</v>
+      </c>
+      <c r="E10" t="n">
+        <v>78</v>
+      </c>
+      <c r="F10" t="n">
+        <v>326</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2164</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3494</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1244</v>
+      </c>
+      <c r="J10" t="n">
+        <v>487</v>
+      </c>
+      <c r="K10" t="n">
+        <v>693</v>
+      </c>
+      <c r="L10" t="n">
+        <v>953</v>
+      </c>
+      <c r="M10" t="n">
+        <v>4535</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1198</v>
+      </c>
+      <c r="O10" t="n">
+        <v>3337</v>
+      </c>
+      <c r="P10" t="n">
+        <v>979</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>89</v>
+      </c>
+      <c r="R10" t="n">
+        <v>40645</v>
+      </c>
+      <c r="S10" t="n">
+        <v>40645</v>
+      </c>
+      <c r="T10" t="n">
+        <v>890000000</v>
+      </c>
+      <c r="U10" t="n">
+        <v>11535</v>
+      </c>
+      <c r="V10" t="n">
+        <v>20777</v>
+      </c>
+      <c r="W10" t="n">
+        <v>4062</v>
+      </c>
+      <c r="X10" t="n">
+        <v>1068</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>28184</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>-541</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>8244</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>50024</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>5694</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>5001</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0.1835</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0.0622</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>-0.0455</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>10432</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0.1726</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.09420000000000001</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0.0827</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>0.0552</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>1043</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>57.96</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>14.88</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>32401</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>50</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>170</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>126</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>0.1543</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="BE10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B11" t="n">
+        <v>87584</v>
+      </c>
+      <c r="C11" t="n">
+        <v>80243</v>
+      </c>
+      <c r="D11" t="n">
+        <v>9936</v>
+      </c>
+      <c r="E11" t="n">
+        <v>87</v>
+      </c>
+      <c r="F11" t="n">
+        <v>375</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2692</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4185</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1581</v>
+      </c>
+      <c r="J11" t="n">
+        <v>450</v>
+      </c>
+      <c r="K11" t="n">
+        <v>826</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1180</v>
+      </c>
+      <c r="M11" t="n">
+        <v>6801</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1728</v>
+      </c>
+      <c r="O11" t="n">
+        <v>5073</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1335</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>89</v>
+      </c>
+      <c r="R11" t="n">
+        <v>60561</v>
+      </c>
+      <c r="S11" t="n">
+        <v>60561</v>
+      </c>
+      <c r="T11" t="n">
+        <v>890000000</v>
+      </c>
+      <c r="U11" t="n">
+        <v>15614</v>
+      </c>
+      <c r="V11" t="n">
+        <v>30621</v>
+      </c>
+      <c r="W11" t="n">
+        <v>6878</v>
+      </c>
+      <c r="X11" t="n">
+        <v>916</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>42743</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>5590</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>14237</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>73461</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>8357</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>7531</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0.4487</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0.4677</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0.5059</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0.5202</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>14123</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0.1613</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0.0954</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>0.07770000000000001</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>0.0579</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>992</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>88.29000000000001</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>12.73</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>46324</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>4</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>59</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>178</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>123</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>0.1626</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="BE11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BF11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>era</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>avg_sales_growth</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>avg_ebitda_margin</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>avg_roce</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>avg_ccc</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>avg_debt_to_ebitda</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>COVID</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.0462</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.0983</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1548</v>
+      </c>
+      <c r="E2" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pre-COVID</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.2213</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0969</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.2039</v>
+      </c>
+      <c r="E3" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.2667</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.3261</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1059</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.1785</v>
+      </c>
+      <c r="E4" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -11829,10 +14033,6 @@
       <c r="AD2" t="n">
         <v>1053.37</v>
       </c>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="n">
         <v>2654.82</v>
       </c>
@@ -11851,8 +14051,6 @@
       <c r="AN2" t="n">
         <v>0.0537</v>
       </c>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="n">
         <v>2.69</v>
       </c>
@@ -11868,14 +14066,12 @@
       <c r="AU2" t="n">
         <v>2.17</v>
       </c>
-      <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>63</v>
       </c>
       <c r="AX2" t="n">
         <v>136</v>
       </c>
-      <c r="AY2" t="inlineStr"/>
       <c r="AZ2" t="n">
         <v>0.1723</v>
       </c>

</xml_diff>

<commit_message>
Week3: SQL analysis, multi-company schema, fixed debt column + partition bugs
</commit_message>
<xml_diff>
--- a/data/TITAN PROJECT.xlsx
+++ b/data/TITAN PROJECT.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Sheet1" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Week2 Pipeline" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Week2 Era Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="SQL Output" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="IQ_CH">110000</definedName>
@@ -1320,10 +1321,6 @@
       <c r="AD2" t="n">
         <v>1053.37</v>
       </c>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="n">
         <v>2654.82</v>
       </c>
@@ -1342,8 +1339,6 @@
       <c r="AN2" t="n">
         <v>0.0537</v>
       </c>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="n">
         <v>2.69</v>
       </c>
@@ -1359,14 +1354,12 @@
       <c r="AU2" t="n">
         <v>2.17</v>
       </c>
-      <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="n">
         <v>63</v>
       </c>
       <c r="AX2" t="n">
         <v>136</v>
       </c>
-      <c r="AY2" t="inlineStr"/>
       <c r="AZ2" t="n">
         <v>0.1723</v>
       </c>
@@ -3123,6 +3116,744 @@
       </c>
       <c r="F4" t="n">
         <v>2.86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>company_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fiscal_year</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ebitda_margin</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>debt</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>capital_employed</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cash_conversion_cycle</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>roce</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>roce_change_pct</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>roce_rank</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>roce_quartile</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2014</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1497</v>
+      </c>
+      <c r="D2" t="n">
+        <v>60642.28</v>
+      </c>
+      <c r="E2" t="n">
+        <v>126245.73</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>0.1883</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1491</v>
+      </c>
+      <c r="D3" t="n">
+        <v>73610.39</v>
+      </c>
+      <c r="E3" t="n">
+        <v>129872.31</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-92</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1406</v>
+      </c>
+      <c r="D4" t="n">
+        <v>69359.96000000001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>148312.37</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-92</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.1462</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-5.28</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.1097</v>
+      </c>
+      <c r="D5" t="n">
+        <v>78603.98</v>
+      </c>
+      <c r="E5" t="n">
+        <v>136665.87</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-118</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.08550000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-6.07</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.1079</v>
+      </c>
+      <c r="D6" t="n">
+        <v>88950.47</v>
+      </c>
+      <c r="E6" t="n">
+        <v>184378.38</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-105</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0537</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-3.18</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.08169999999999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>106175.34</v>
+      </c>
+      <c r="E7" t="n">
+        <v>166354.9</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-97</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-4.72</v>
+      </c>
+      <c r="I7" t="n">
+        <v>8</v>
+      </c>
+      <c r="J7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0689</v>
+      </c>
+      <c r="D8" t="n">
+        <v>124787.64</v>
+      </c>
+      <c r="E8" t="n">
+        <v>186998.67</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-113</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.0184</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-2.49</v>
+      </c>
+      <c r="I8" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.1293</v>
+      </c>
+      <c r="D9" t="n">
+        <v>142130.57</v>
+      </c>
+      <c r="E9" t="n">
+        <v>197377.29</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-141</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0443</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0888</v>
+      </c>
+      <c r="D10" t="n">
+        <v>146449.03</v>
+      </c>
+      <c r="E10" t="n">
+        <v>191010.27</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-119</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-4.49</v>
+      </c>
+      <c r="I10" t="n">
+        <v>9</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="D11" t="n">
+        <v>134113.44</v>
+      </c>
+      <c r="E11" t="n">
+        <v>179435.23</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-106</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0388</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="I11" t="n">
+        <v>7</v>
+      </c>
+      <c r="J11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0878</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1882.43</v>
+      </c>
+      <c r="E12" t="n">
+        <v>6114.81</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>0.1723</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>7</v>
+      </c>
+      <c r="J12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1691.01</v>
+      </c>
+      <c r="E13" t="n">
+        <v>6780.89</v>
+      </c>
+      <c r="F13" t="n">
+        <v>78</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.2231</v>
+      </c>
+      <c r="H13" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.1008</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2392.98</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8463.129999999999</v>
+      </c>
+      <c r="F14" t="n">
+        <v>77</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.2163</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3562</v>
+      </c>
+      <c r="E15" t="n">
+        <v>10231</v>
+      </c>
+      <c r="F15" t="n">
+        <v>89</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.2067</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="I15" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.07969999999999999</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5638</v>
+      </c>
+      <c r="E16" t="n">
+        <v>13135</v>
+      </c>
+      <c r="F16" t="n">
+        <v>92</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.1028</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-10.39</v>
+      </c>
+      <c r="I16" t="n">
+        <v>10</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.1161</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7275</v>
+      </c>
+      <c r="E17" t="n">
+        <v>16578</v>
+      </c>
+      <c r="F17" t="n">
+        <v>120</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="I17" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1203</v>
+      </c>
+      <c r="D18" t="n">
+        <v>9367</v>
+      </c>
+      <c r="E18" t="n">
+        <v>21218</v>
+      </c>
+      <c r="F18" t="n">
+        <v>103</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.2093</v>
+      </c>
+      <c r="H18" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.1036</v>
+      </c>
+      <c r="D19" t="n">
+        <v>15528</v>
+      </c>
+      <c r="E19" t="n">
+        <v>24921</v>
+      </c>
+      <c r="F19" t="n">
+        <v>95</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.1889</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-2.04</v>
+      </c>
+      <c r="I19" t="n">
+        <v>5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.09420000000000001</v>
+      </c>
+      <c r="D20" t="n">
+        <v>20777</v>
+      </c>
+      <c r="E20" t="n">
+        <v>32401</v>
+      </c>
+      <c r="F20" t="n">
+        <v>126</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.1543</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-3.46</v>
+      </c>
+      <c r="I20" t="n">
+        <v>9</v>
+      </c>
+      <c r="J20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.0954</v>
+      </c>
+      <c r="D21" t="n">
+        <v>30621</v>
+      </c>
+      <c r="E21" t="n">
+        <v>46324</v>
+      </c>
+      <c r="F21" t="n">
+        <v>123</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.1626</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="I21" t="n">
+        <v>8</v>
+      </c>
+      <c r="J21" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week5: sensitivity, Monte Carlo, driver ranking - WACC is #1 driver
</commit_message>
<xml_diff>
--- a/data/TITAN PROJECT.xlsx
+++ b/data/TITAN PROJECT.xlsx
@@ -21,6 +21,7 @@
     <sheet name="Week2 Era Summary" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="SQL Output" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Assumptions" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Sensitivity_Summary" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="IQ_CH">110000</definedName>
@@ -4165,6 +4166,87 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Week 5 - Sensitivity Analysis Summary (Titan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Finding</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WACC x Terminal Growth spread</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Rs.1051.62 to Rs.3867.55 (3.7x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Growth x Margin range</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rs.1250.40 to Rs.4862.42 (0 negative cells)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Monte Carlo median value/share</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Rs.2882.35 (P5=2226.83, P95=4309.70), 0.0% negative-equity probability</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Most impactful assumption</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>wacc - Rs.1602.86 (58.0% of base)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>